<commit_message>
Add feature to show inconsistent boxes
</commit_message>
<xml_diff>
--- a/projects/kartgenerator/assets/examples/exempel.xlsx
+++ b/projects/kartgenerator/assets/examples/exempel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ledka\ledkarlsson.github.io\projects\kartgenerator\assets\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0187DF-91B5-4131-A029-4E5860AC6B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89122203-B76A-4C27-8732-B307FB8B1CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2565" yWindow="6540" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2880" yWindow="2880" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rapport" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>Område/plats</t>
   </si>
@@ -74,6 +74,15 @@
   </si>
   <si>
     <t>Josefinsson</t>
+  </si>
+  <si>
+    <t>Brygga B - 54</t>
+  </si>
+  <si>
+    <t>Brygga B - 55</t>
+  </si>
+  <si>
+    <t>Brygga B - 56</t>
   </si>
 </sst>
 </file>
@@ -128,9 +137,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -168,7 +177,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -274,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -416,7 +425,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -427,7 +436,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
@@ -518,6 +527,21 @@
       </c>
       <c r="E5" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>